<commit_message>
revert changes in Definition sheet
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/methanol/Model_Data_Base_methanol_updated.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/methanol/Model_Data_Base_methanol_updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\methanol\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kar.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\methanol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CEE26B4-C3EC-4C15-8E85-F994C6B0F0A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D32D38A-1944-4AA6-BCF9-E2D9BADB1045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-10110" yWindow="-21720" windowWidth="51840" windowHeight="21120" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="0" yWindow="390" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -1705,14 +1705,14 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{576C757C-091A-46DF-949E-B17661031FDE}">
   <dimension ref="A1:R12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="13.77734375" customWidth="1"/>
-    <col min="2" max="2" width="19.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="18" width="10.5546875" customWidth="1"/>
+    <col min="1" max="1" width="13.7109375" customWidth="1"/>
+    <col min="2" max="2" width="19.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="18" width="10.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1768,7 +1768,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>69</v>
       </c>
@@ -1781,7 +1781,7 @@
       <c r="P2" s="1"/>
       <c r="Q2" s="1"/>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>109</v>
       </c>
@@ -1794,7 +1794,7 @@
       <c r="P3" s="1"/>
       <c r="Q3" s="1"/>
     </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>110</v>
       </c>
@@ -1807,7 +1807,7 @@
       <c r="P4" s="1"/>
       <c r="Q4" s="1"/>
     </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>89</v>
       </c>
@@ -1829,7 +1829,7 @@
       <c r="P5" s="1"/>
       <c r="Q5" s="1"/>
     </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>85</v>
       </c>
@@ -1842,7 +1842,7 @@
       <c r="P6" s="1"/>
       <c r="Q6" s="1"/>
     </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>84</v>
       </c>
@@ -1859,7 +1859,7 @@
         <v>20.192799999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>83</v>
       </c>
@@ -1896,7 +1896,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>77</v>
       </c>
@@ -1912,7 +1912,7 @@
       <c r="P9" s="1"/>
       <c r="Q9" s="1"/>
     </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>115</v>
       </c>
@@ -1925,7 +1925,7 @@
       <c r="P10" s="1"/>
       <c r="Q10" s="1"/>
     </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>117</v>
       </c>
@@ -1938,7 +1938,7 @@
       <c r="P11" s="1"/>
       <c r="Q11" s="1"/>
     </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>94</v>
       </c>
@@ -1981,14 +1981,15 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CABA7C5-6230-4207-9D35-0A95D86E66AC}">
   <dimension ref="A1:Q12"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.6640625" customWidth="1"/>
-    <col min="2" max="2" width="13.21875" customWidth="1"/>
-    <col min="7" max="8" width="9.77734375" customWidth="1"/>
+    <col min="1" max="1" width="14.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.28515625" customWidth="1"/>
+    <col min="7" max="7" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
@@ -2041,7 +2042,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
         <v>69</v>
       </c>
@@ -2066,7 +2067,7 @@
       <c r="P2" s="7"/>
       <c r="Q2" s="7"/>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A3" s="4" t="s">
         <v>109</v>
       </c>
@@ -2091,7 +2092,7 @@
       <c r="P3" s="4"/>
       <c r="Q3" s="4"/>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>110</v>
       </c>
@@ -2116,7 +2117,7 @@
       <c r="P4" s="3"/>
       <c r="Q4" s="3"/>
     </row>
-    <row r="5" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="4" t="s">
         <v>89</v>
       </c>
@@ -2151,7 +2152,7 @@
       <c r="P5" s="4"/>
       <c r="Q5" s="4"/>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A6" s="3" t="s">
         <v>85</v>
       </c>
@@ -2184,7 +2185,7 @@
       <c r="P6" s="3"/>
       <c r="Q6" s="3"/>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A7" s="4" t="s">
         <v>84</v>
       </c>
@@ -2218,7 +2219,7 @@
       <c r="P7" s="4"/>
       <c r="Q7" s="4"/>
     </row>
-    <row r="8" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>83</v>
       </c>
@@ -2256,7 +2257,7 @@
       <c r="P8" s="3"/>
       <c r="Q8" s="3"/>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
         <v>77</v>
       </c>
@@ -2289,7 +2290,7 @@
       <c r="P9" s="4"/>
       <c r="Q9" s="4"/>
     </row>
-    <row r="10" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>94</v>
       </c>
@@ -2320,7 +2321,7 @@
       <c r="P10" s="6"/>
       <c r="Q10" s="6"/>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
         <v>115</v>
       </c>
@@ -2349,7 +2350,7 @@
       <c r="P11" s="4"/>
       <c r="Q11" s="4"/>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>117</v>
       </c>
@@ -2402,33 +2403,34 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C870BDA0-9E4C-481D-87BE-9D47789809C8}">
   <dimension ref="A1:AA11"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" customWidth="1"/>
-    <col min="2" max="2" width="19.5546875" customWidth="1"/>
-    <col min="3" max="6" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="35.21875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="15.21875" customWidth="1"/>
-    <col min="9" max="9" width="17.44140625" customWidth="1"/>
-    <col min="10" max="10" width="15.44140625" customWidth="1"/>
-    <col min="11" max="11" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="15.44140625" customWidth="1"/>
+    <col min="1" max="1" width="27.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="5" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="15.28515625" customWidth="1"/>
+    <col min="9" max="9" width="17.42578125" customWidth="1"/>
+    <col min="10" max="10" width="15.42578125" customWidth="1"/>
+    <col min="11" max="11" width="17.42578125" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="15.42578125" customWidth="1"/>
     <col min="13" max="13" width="19" customWidth="1"/>
-    <col min="14" max="14" width="15.44140625" customWidth="1"/>
+    <col min="14" max="14" width="15.42578125" customWidth="1"/>
     <col min="15" max="15" width="19" customWidth="1"/>
-    <col min="16" max="16" width="10.5546875" customWidth="1"/>
-    <col min="17" max="17" width="15.5546875" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="17.21875" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="18.77734375" bestFit="1" customWidth="1"/>
-    <col min="20" max="20" width="18.77734375" customWidth="1"/>
-    <col min="21" max="21" width="12.77734375" customWidth="1"/>
-    <col min="22" max="23" width="17.77734375" bestFit="1" customWidth="1"/>
-    <col min="24" max="25" width="19.44140625" bestFit="1" customWidth="1"/>
-    <col min="26" max="26" width="35.21875" bestFit="1" customWidth="1"/>
-    <col min="27" max="27" width="24.21875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="10.5703125" customWidth="1"/>
+    <col min="17" max="17" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="17.28515625" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="18.7109375" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="18.7109375" customWidth="1"/>
+    <col min="21" max="21" width="12.7109375" customWidth="1"/>
+    <col min="22" max="23" width="17.7109375" bestFit="1" customWidth="1"/>
+    <col min="24" max="25" width="19.42578125" bestFit="1" customWidth="1"/>
+    <col min="26" max="26" width="35.28515625" bestFit="1" customWidth="1"/>
+    <col min="27" max="27" width="24.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>27</v>
       </c>
@@ -2511,7 +2513,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>71</v>
       </c>
@@ -2570,7 +2572,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>88</v>
       </c>
@@ -2626,7 +2628,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="4" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>90</v>
       </c>
@@ -2682,7 +2684,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="5" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>73</v>
       </c>
@@ -2720,7 +2722,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>122</v>
       </c>
@@ -2779,7 +2781,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>123</v>
       </c>
@@ -2817,7 +2819,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>124</v>
       </c>
@@ -2876,7 +2878,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>125</v>
       </c>
@@ -2914,7 +2916,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>126</v>
       </c>
@@ -2973,7 +2975,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="11" spans="1:27" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:27" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>127</v>
       </c>
@@ -2990,6 +2992,15 @@
         <v>32</v>
       </c>
       <c r="H11">
+        <v>1000</v>
+      </c>
+      <c r="I11">
+        <v>1000</v>
+      </c>
+      <c r="L11">
+        <v>1000</v>
+      </c>
+      <c r="M11">
         <v>1000</v>
       </c>
       <c r="T11">
@@ -3027,22 +3038,22 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{981CFA5E-60F3-446F-A856-2FA65B76879A}">
   <dimension ref="A1:K3"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.44140625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="16.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.77734375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.77734375" customWidth="1"/>
-    <col min="8" max="8" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.5703125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="8" max="8" width="12.7109375" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="11" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="18.21875" customWidth="1"/>
+    <col min="10" max="10" width="11.28515625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="18.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>33</v>
       </c>
@@ -3077,7 +3088,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>79</v>
       </c>
@@ -3103,7 +3114,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>80</v>
       </c>
@@ -3158,102 +3169,102 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{71DC79B9-9C58-497E-9FD8-D3F2239E9BDC}">
   <dimension ref="A1:A19"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="3" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="4" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="6" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="7" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>47</v>
       </c>
     </row>
-    <row r="8" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="9" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>48</v>
       </c>
     </row>
-    <row r="10" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="11" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="12" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="13" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>51</v>
       </c>
     </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="15" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="16" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>68</v>
       </c>
     </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="19" spans="1:1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>95</v>
       </c>

</xml_diff>

<commit_message>
- changed the typo in 01_input_raw (ofshore to offshore) - applied new changes to 'Object__to_from_node_definition' sheet - appled new changes to 'Object__to_from_node' sheet *Object__to_from_node* requires PPA conditioning*
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/methanol/Model_Data_Base_methanol_updated.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/methanol/Model_Data_Base_methanol_updated.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kar.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\methanol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D32D38A-1944-4AA6-BCF9-E2D9BADB1045}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02EA1C38-4C41-4541-80E6-E63C9685B111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="390" windowWidth="28800" windowHeight="15345" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="5070" yWindow="5070" windowWidth="38700" windowHeight="15345" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>
@@ -457,7 +457,7 @@
     <t>pl_wholesale_wind_offshore</t>
   </si>
   <si>
-    <t>pl_wind_ofshore_PPA</t>
+    <t>pl_wind_offshore_PPA</t>
   </si>
 </sst>
 </file>

</xml_diff>

<commit_message>
created '_updated' files for all products
</commit_message>
<xml_diff>
--- a/Spine_Projects/01_input_data/01_input_raw/Products/methanol/Model_Data_Base_methanol_updated.xlsx
+++ b/Spine_Projects/01_input_data/01_input_raw/Products/methanol/Model_Data_Base_methanol_updated.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kar.eco\Documents\GitHub\Nord_H2ub\Spine_Projects\01_input_data\01_input_raw\Products\methanol\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{02EA1C38-4C41-4541-80E6-E63C9685B111}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976B75BF-2265-4260-B68E-9D163759AD3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5070" yWindow="5070" windowWidth="38700" windowHeight="15345" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="26010" windowHeight="20985" activeTab="2" xr2:uid="{50334894-9481-4F8E-BD29-206032E10C62}"/>
   </bookViews>
   <sheets>
     <sheet name="Units" sheetId="1" r:id="rId1"/>

</xml_diff>